<commit_message>
chore: back up verified 2026H1 AI chain delta
</commit_message>
<xml_diff>
--- a/watchlists/AI产业链.xlsx
+++ b/watchlists/AI产业链.xlsx
@@ -1152,7 +1152,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>高速光模块</t>
@@ -1170,16 +1170,16 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>通过收购索尔思切入光模块（含光芯片），年报确认100G/200G PAM4 EML与10G-1.6T模块矩阵，同时有AI PCB协同；主板块由光芯片降为高速光模块，AI PCB放备注跟踪，风险是并购整合、负债和客户放量节奏。证据A。</t>
+          <t>2026H1正式中报（未经审计）：营收277.98亿元、归母29.57亿元、经营现金流23.84亿元（同比-4.65%）；光模块收入53.51亿元、毛利率39.33%；应收/存货105.98/114.18亿元，年初97.93/89.29亿元。高端AI PCB项目预算70亿元、进度27.02%；光模块产线预算18亿元、82.61%；泰国PCB/光模块配套预算13.12亿元、88.37%，均未视为投产/订单/收入。客户、订单、光芯片/AI PCB独立收入与毛利及认证范围=evidence_absent。证据A：CNINFO 2026-08-22。</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>已处理</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
+          <t>已处理；2026-08-22正式中报复核（未经审计）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>高速光模块</t>
@@ -1197,12 +1197,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>全球高速光模块龙头，2025年营收382.40亿元、归母净利107.97亿元，高速光模块、800G/1.6T放量已兑现；主板块保留高速光模块，风险是估值拥挤、客户集中、年降和物料约束。证据A。</t>
+          <t>2026H1正式中报（未经审计）：营收417.78亿元、归母136.51亿元、经营现金流18.00亿元（同比-44.08%）；光通信收发模块收入413.55亿元、毛利率46.59%；应收/存货150.01/198.26亿元，年初62.77/126.81亿元。800G/1.6T/硅光的客户、订单、独立收入/毛利及认证范围=evidence_absent。证据A：CNINFO 2026-08-22。</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-08-22正式中报复核（未经审计）</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="60" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>新型光纤</t>
@@ -2126,12 +2126,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20更新：主营仍是“光棒—光纤—光缆”光传输产品。2025年光传输产品收入83.46亿元、占58.56%、毛利率35.90%；光互联组件收入31.44亿元、占22.06%、毛利率39.73%。2026H1预告归母净利润24—30亿元（同比+711%—914%）、扣非20—26亿元（同比+1349%—1784%）；据Q1归母4.95亿元推算，Q2归母约19.05—25.05亿元。公司称增量来自算力数据中心加速建设、国内外新型光纤光缆需求、核心客户拓展、产品结构优化及盈利能力提升。产品层：普通单模、预制棒及光缆仍是量的基本盘；G.654.E已超百万芯公里规模部署，OM4/OM4 Pro/OM5已规模商用；G.657.A2为成熟量产品种且对本轮高端光棒涨价敏感，但公司未披露其独立收入、ASP或毛利率；空芯/多芯仍偏产业化导入，不能视为当前利润主体。价格基准判断：A2及高端光棒2026H2仍偏强，2027H1涨幅钝化，名义高点更可能在2027Q2—Q3，2027H2—2028随有效产能释放而分化、回落风险上升。证据边界：行业A2报价及Corning海外长协不等于长飞实现售价、客户或订单；继续跟踪2026中报分产品收入/毛利率、现金流、存货及客户订单。来源：公司2026H1业绩预增公告、2025年报、2026-05-22业绩说明会；行业价格为二级证据。</t>
+          <t>2026H1正式中报（未经审计）：营收98.09亿元、归母29.25亿元、经营现金流18.26亿元；光传输/光互联组件收入约61.26/22.38亿元、毛利率63.11%/48.97%；应收/存货72.70/44.70亿元，年初59.50/31.53亿元。PMF/CPO及空芯光纤的客户、订单、独立收入/毛利及认证范围=evidence_absent。证据A：上交所2026-08-22。</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>已处理；2026-06-28 光纤上游补充</t>
+          <t>已处理；2026-08-22正式中报复核（未经审计）</t>
         </is>
       </c>
     </row>
@@ -3134,7 +3134,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="36" customHeight="1">
+    <row r="76" ht="75" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
           <t>高端高速铜箔</t>
@@ -3152,12 +3152,12 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>PCB级RTF/HVLP进展最直接，年报披露RTF-3/4认证并批量供货、HVLP1-3批量供货、HVLP4小规模放量、HVLP5完成样品认证并推进导入；主板块由高端铜箔细化为HVLP铜箔，风险是HVLP5多客户、收入和毛利率仍需量化。证据A/B。 2026-06-17 HVLP4/T-glass复核：放“交易弹性/条件式HVLP期权”；HVLP4/5从纯watch提高到watch_to_soft验证优先级，但需多客户批量、加工费、电子电路铜箔收入占比和毛利证据，不能混同锂电铜箔修复；官方追杀后，NVIDIA锁产/寄售/LTA/prepayment仍未闭环。</t>
+          <t>2026H1正式中报（未经审计）：营收91.97亿元、归母2.63亿元、经营现金流-6.13亿元；电子电路铜箔收入13.08亿元、毛利率4.85%；应收/存货35.84/26.80亿元，年初34.44/18.72亿元。H1启动5万吨AI高端电子电路铜箔项目（完全达产后年产5万吨为规划，非已达产）。HVLP/RTF/载体铜箔的客户、订单、独立收入/毛利及认证范围=evidence_absent。证据A：CNINFO 2026-08-22。</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>已处理；2026-06-17证据分层；2026-06-17官方锁产追杀仍未闭环</t>
+          <t>已处理；2026-08-22正式中报复核（未经审计）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: correct AI chain code and refresh concentration metadata
</commit_message>
<xml_diff>
--- a/watchlists/AI产业链.xlsx
+++ b/watchlists/AI产业链.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI产业链" sheetId="1" r:id="Ra745c65ac7ac4598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI产业链" sheetId="1" r:id="Rd1f8d500f6a04c04"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7404,10 +7404,8 @@
           <x:t xml:space="preserve">半导体测试服务</x:t>
         </x:is>
       </x:c>
-      <x:c r="B241" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">430139</x:t>
-        </x:is>
+      <x:c r="B241" s="3" t="str">
+        <x:v>920139</x:v>
       </x:c>
       <x:c r="C241" s="2" t="inlineStr">
         <x:is>
@@ -11526,6 +11524,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd72c834f64724eb1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cd08c757d024d8b"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
data: update changyingtong AI-chain evidence
</commit_message>
<xml_diff>
--- a/watchlists/AI产业链.xlsx
+++ b/watchlists/AI产业链.xlsx
@@ -1606,7 +1606,7 @@
     <row r="26" ht="90" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>FAU</t>
+          <t>新型光纤/无源内连光器件</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1621,12 +1621,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>并表子公司生一升的无源内连光器件覆盖AWG、MT-FA/FA-REC、光纤阵列；2026H1正式披露用于100G–800G高速光模块、数据中心/云计算，且无源内连产品交付增加。1.6T MT-FA+Lens项目已完成工艺研发并称实现产品量产，但未披露CPO客户、订单、出货或独立收入。重点复核：器件保偏光纤仅处客户验证，公司称其适配CPO/硅光互连；2026-08-15公告称业务体量有限、在手订单少、通信领域未新增重大客户，不能按CPO规模应用、AI订单或收入处理。证据A：上交所2026-08-15、2026-08-25。</t>
+          <t>2026H1官方：无源内连光器件需求增加；器件级保偏光纤（PMF）面向AI服务器/智算集群，披露称匹配CPO/硅光；“FAU型器件保偏光纤”只列为FAU多芯阵列应用。CPO、PMF、PM-FAU均为条件性观察（产品方向/验证与产能表述，非商业闭环）；具名客户、CPO/PMF/PM-FAU量产订单、独立AI收入均=evidence_absent。证据A：上交所《2026年半年度报告》2026-08-25。</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>新增；2026-08-31重点复核：无源内连=收入，器件保偏=验证/观察</t>
+          <t>已复核；2026H1官方披露；条件性观察（CPO/PMF/PM-FAU），客户/订单/独立AI收入=evidence_absent</t>
         </is>
       </c>
     </row>

</xml_diff>